<commit_message>
Quellenbasis: die zwei offenen Zeilen aufgeloest, keine offen mehr
Nr 4 und Nr 133 waren nicht ungeklaert, sie standen im Register selbst.
Die Spalte Herausgeber / Institution nennt Steinmueller 2012 und
Zukunftsinstitut (Horx) 2021. Der automatische Abgleich hatte nur den
Titel ausgewertet.

  4    -> ZF/2024/Steinmueller-ZF.pdf
  133  -> ZF/2021/Zukunftsinstitut-2021.pdf

Nr 4 zusaetzlich gestuetzt durch foresight Master,
2026-08-18_Grundrisse-der-Zukunft_v1.html: Startfassung nach Steinmueller.

Stand jetzt: geprueft 13, sicher 80, wahrscheinlich 43, offen 0.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KnhC4MKPSYPLr5Crt2DXix
</commit_message>
<xml_diff>
--- a/register/2026-09-03_Grundrisse_Foresight-Register_2045_v15.xlsx
+++ b/register/2026-09-03_Grundrisse_Foresight-Register_2045_v15.xlsx
@@ -1486,9 +1486,14 @@
           <t>verifiziert</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ZF/2024/Steinmüller-ZF.pdf</t>
+        </is>
+      </c>
       <c r="L5" s="54" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>geprüft</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2746,7 @@
           <t>verifiziert</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K26" s="54" t="inlineStr">
         <is>
           <t>Geschichte/Kollaps - Weltreichefpos-02-568704.pdf</t>
         </is>
@@ -2861,7 +2866,7 @@
           <t>verifiziert (Exec Summary geprüft)</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K28" s="54" t="inlineStr">
         <is>
           <t>ZF/2024/CIA Globale Trends 2040/</t>
         </is>
@@ -3521,7 +3526,7 @@
           <t>verifiziert</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="K39" s="54" t="inlineStr">
         <is>
           <t>RK/WBGU/wbgu_jg2011.pdf</t>
         </is>
@@ -3641,7 +3646,7 @@
           <t>verifiziert</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K41" s="54" t="inlineStr">
         <is>
           <t>Stadt/2016/wbgu_Städte_hg2016-hoch.pdf</t>
         </is>
@@ -4001,7 +4006,7 @@
           <t>verifiziert</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K47" s="54" t="inlineStr">
         <is>
           <t>Umwelt/SDGs_2016/sdg_index_and_dashboards_compact.pdf</t>
         </is>
@@ -4061,7 +4066,7 @@
           <t>verifiziert</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="K48" s="54" t="inlineStr">
         <is>
           <t>Umwelt/2018/uba_texte_89_2018_vorsorgeorientierte_postwachstumsposition.pdf</t>
         </is>
@@ -4121,7 +4126,7 @@
           <t>verifiziert</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="K49" s="54" t="inlineStr">
         <is>
           <t>the Future/Null-Wachstums Paper -2016.pdf</t>
         </is>
@@ -4181,7 +4186,7 @@
           <t>verifiziert (4-S.-Artikel)</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="K50" s="54" t="inlineStr">
         <is>
           <t>Wissen/5924_Schneidewind.pdf</t>
         </is>
@@ -4961,7 +4966,7 @@
           <t>verifiziert</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr">
+      <c r="K63" s="54" t="inlineStr">
         <is>
           <t>Innovation/2024/TAB-Risikobericht_.pdf</t>
         </is>
@@ -5741,7 +5746,7 @@
           <t>verifiziert (Werk)</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr">
+      <c r="K76" s="54" t="inlineStr">
         <is>
           <t>Co-evolution/Essay -co-evoution_Roadmap bis 2100.docx</t>
         </is>
@@ -6701,7 +6706,7 @@
           <t>verifiziert</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr">
+      <c r="K92" s="54" t="inlineStr">
         <is>
           <t>Wirtschaft/Milanovic_WPS6719_Elephant.pdf</t>
         </is>
@@ -9041,9 +9046,14 @@
           <t>verifiziert</t>
         </is>
       </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>ZF/2021/Zukunftsinstitut-2021.pdf</t>
+        </is>
+      </c>
       <c r="L134" s="54" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>geprüft</t>
         </is>
       </c>
     </row>
@@ -9096,7 +9106,7 @@
           <t>verifiziert</t>
         </is>
       </c>
-      <c r="K135" t="inlineStr">
+      <c r="K135" s="54" t="inlineStr">
         <is>
           <t>ZF/Zukunftsräte/jonathan-boston-lecture-american-university.pdf</t>
         </is>
@@ -9336,7 +9346,7 @@
           <t>verifiziert</t>
         </is>
       </c>
-      <c r="K139" t="inlineStr">
+      <c r="K139" s="54" t="inlineStr">
         <is>
           <t>ZdA/2021/2021-OECD-ZdA-KI-7c895724-en.pdf</t>
         </is>

</xml_diff>